<commit_message>
Leads: 2026-10-17 03:58 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Horizon Heating &amp; Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>horizonheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.horizonheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cleanliness Vivian</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>joe@horizonoc.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>714-577-8220</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>furnace repair Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 04:01 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,126 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tesson Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tessonroofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://tessonroofing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Louis County</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>support@tessonroofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(314) 932-1042</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofer St Louis MO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Helsley Roofing Company</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>helsleyroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://helsleyroofing.com/service-areas/richardson-tx-roofers/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Alan Helsley</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@helsleyroofing.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(972) 578-8982</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>residential roofing company Richardson TX</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 04:05 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Koon Roofing and Restoration</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>koonroofing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.koonroofing.com/services/roofing-contractor/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Little Ro</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>koon2k7@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(501) 326-2694</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>residential roofing company Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 15:24 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -863,6 +863,62 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Neu Flo Plumbing | Plumber in Buffalo, NY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>neufloplumbing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.neufloplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>daniel.neuman@neufloplumbing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(716) 249-1993</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Buffalo NY</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>plumber Buffalo NY</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 15:26 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -884,7 +884,6 @@
           <t>https://www.neufloplumbing.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>daniel.neuman@neufloplumbing.com</t>
@@ -914,6 +913,66 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mackenzie and Sons Roofing Company</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mackenzieandsonsroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>http://mackenzieandsonsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Energy Star</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>mackenziesons@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(413) 563-9871</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Springfield MA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>84</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof replacement Springfield MA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-17 15:39 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -978,6 +978,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tanks Water Heaters &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>renosparkswaterheaters.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.renosparkswaterheaters.com/services/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Home About</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>tankswaterheatersplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(775) 997-8071</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sparks NV</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>water heater repair Sparks NV</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 15:42 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1038,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A/C Service &amp; Repairs, LLC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>acserviceandrepairs.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://acserviceandrepairs.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Russ Allen</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>russ@acserviceandrepairs.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(817) 737-8423</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>98</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>AC installation Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-17 16:06 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-17.xlsx
+++ b/output/leads_2026-10-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1098,6 +1098,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4everheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.4everheatingandcooling.com/air-conditioning-repair-fremont-california</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Policy Quote</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>support@4everheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(888)884-4927</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>76</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>air conditioning repair Fremont CA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>